<commit_message>
Add scholarship_information column across schema, xlsx, and both web apps
Sits next to academic_requirement in the capture form, CSV export, and
workbook so scholarship/fee-waiver details captured from agency posts
are no longer folded into other_details.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/knowledge_base.xlsx
+++ b/data/knowledge_base.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA1"/>
+  <dimension ref="A1:AB1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -443,6 +443,7 @@
     <col width="22" customWidth="1" min="25" max="25"/>
     <col width="22" customWidth="1" min="26" max="26"/>
     <col width="22" customWidth="1" min="27" max="27"/>
+    <col width="22" customWidth="1" min="28" max="28"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -523,60 +524,65 @@
       </c>
       <c r="P1" t="inlineStr">
         <is>
+          <t>scholarship_information</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
           <t>english_requirement</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>interview_condition</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>initial_deposit</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>application_charge</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>process_duration</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>visa_requirement_notes</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>insurance_cost_estimate</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>travel_cost_estimate</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>cost_of_living_estimate</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>banking_income_requirement</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>application_deadline</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>other_details</t>
         </is>

</xml_diff>